<commit_message>
test(automation): update bug verification tests, add phone country code handling, and enhance Excel reporting with Skipped status validation dropdown
</commit_message>
<xml_diff>
--- a/test-data/QA_Test_Cases.xlsx
+++ b/test-data/QA_Test_Cases.xlsx
@@ -11386,8 +11386,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="I12:I89">
-      <formula1>"Pass,Fail,Not Executed,Blocked"</formula1>
+    <dataValidation type="list" allowBlank="1" sqref="I11:I89">
+      <formula1>"Pass,Fail,Skipped,Not Executed,Blocked"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="L12:L89">
       <formula1>"Critical,High,Medium,Low"</formula1>

</xml_diff>

<commit_message>
docs: remove Newsletter test case from reporting sheets since the feature does not exist in production
</commit_message>
<xml_diff>
--- a/test-data/QA_Test_Cases.xlsx
+++ b/test-data/QA_Test_Cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="598">
   <si>
     <t>Test Case Template for Project</t>
   </si>
@@ -1865,7 +1865,7 @@
     <t/>
   </si>
   <si>
-    <t>■  EXTENDED UI &amp; SEO TESTS  —  Verifying auxiliary features (6 cases)</t>
+    <t>■  EXTENDED UI &amp; SEO TESTS  —  Verifying auxiliary features (5 cases)</t>
   </si>
   <si>
     <t>MTW-EXT-01</t>
@@ -1910,31 +1910,16 @@
     <t>Dropdown opens</t>
   </si>
   <si>
-    <t>MTW-EXT-03</t>
-  </si>
-  <si>
-    <t>Newsletter subscription</t>
-  </si>
-  <si>
-    <t>MTW-TC-57</t>
+    <t>MTW-EXT-04</t>
+  </si>
+  <si>
+    <t>Footer social media links</t>
+  </si>
+  <si>
+    <t>MTW-TC-58</t>
   </si>
   <si>
     <t>User scrolls to footer</t>
-  </si>
-  <si>
-    <t>Test newsletter subscription input</t>
-  </si>
-  <si>
-    <t>Can subscribe</t>
-  </si>
-  <si>
-    <t>MTW-EXT-04</t>
-  </si>
-  <si>
-    <t>Footer social media links</t>
-  </si>
-  <si>
-    <t>MTW-TC-58</t>
   </si>
   <si>
     <t>Test Social Media href links</t>
@@ -2639,7 +2624,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA100"/>
+  <dimension ref="A1:AA99"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.63"/>
   <cols>
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
@@ -7148,19 +7133,19 @@
         <v>586</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>567</v>
+        <v>587</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>582</v>
+        <v>589</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="G98" s="1" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="H98" s="1" t="s">
         <v>563</v>
@@ -7175,30 +7160,30 @@
         <v>563</v>
       </c>
       <c r="L98" s="1" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>594</v>
+        <v>589</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="G99" s="1" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="H99" s="1" t="s">
         <v>563</v>
@@ -7213,44 +7198,6 @@
         <v>563</v>
       </c>
       <c r="L99" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A100" s="1" t="s">
-        <v>597</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>599</v>
-      </c>
-      <c r="D100" s="1" t="s">
-        <v>600</v>
-      </c>
-      <c r="E100" s="1" t="s">
-        <v>594</v>
-      </c>
-      <c r="F100" s="1" t="s">
-        <v>601</v>
-      </c>
-      <c r="G100" s="1" t="s">
-        <v>602</v>
-      </c>
-      <c r="H100" s="1" t="s">
-        <v>563</v>
-      </c>
-      <c r="I100" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="J100" s="1" t="s">
-        <v>572</v>
-      </c>
-      <c r="K100" s="1" t="s">
-        <v>563</v>
-      </c>
-      <c r="L100" s="1" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>